<commit_message>
Seguimiento de cuentas · LS · 2026-08-11 22:40
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G600"/>
+  <dimension ref="A1:G601"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19517,6 +19517,35 @@
         </is>
       </c>
       <c r="G600" t="inlineStr"/>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>Comitente</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>Allaria Alyc</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Novus Dolar MM</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr"/>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>Abierta</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>Ok para operar.</t>
+        </is>
+      </c>
+      <c r="G601" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24406,7 +24435,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Fondo</t>
+          <t>FCI</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">

</xml_diff>

<commit_message>
Seguimiento de cuentas · LS · 2026-08-19 14:53
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -18,7 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -48,8 +51,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -8194,7 +8198,11 @@
           <t>Pedido de apertura</t>
         </is>
       </c>
-      <c r="G242" t="inlineStr"/>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>19/08 consulta estado</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -17463,7 +17471,11 @@
           <t>Pedido de apertura</t>
         </is>
       </c>
-      <c r="G535" t="inlineStr"/>
+      <c r="G535" t="inlineStr">
+        <is>
+          <t>19/08 consulta estado</t>
+        </is>
+      </c>
     </row>
     <row r="536">
       <c r="A536" t="inlineStr">
@@ -19599,10 +19611,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-06-17</t>
-        </is>
+      <c r="A2" s="1" t="n">
+        <v>45825</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -19632,10 +19642,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-06-17</t>
-        </is>
+      <c r="A3" s="1" t="n">
+        <v>45825</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -19665,10 +19673,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-06-17</t>
-        </is>
+      <c r="A4" s="1" t="n">
+        <v>45825</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -19698,10 +19704,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-06-17</t>
-        </is>
+      <c r="A5" s="1" t="n">
+        <v>45825</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -19731,10 +19735,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-04-21</t>
-        </is>
+      <c r="A6" s="1" t="n">
+        <v>46133</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -19764,10 +19766,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2025-06-19</t>
-        </is>
+      <c r="A7" s="1" t="n">
+        <v>45827</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -19797,10 +19797,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2025-06-12</t>
-        </is>
+      <c r="A8" s="1" t="n">
+        <v>45820</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -19830,10 +19828,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2025-06-24</t>
-        </is>
+      <c r="A9" s="1" t="n">
+        <v>45832</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -19863,10 +19859,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2025-06-24</t>
-        </is>
+      <c r="A10" s="1" t="n">
+        <v>45832</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -19896,10 +19890,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2025-06-24</t>
-        </is>
+      <c r="A11" s="1" t="n">
+        <v>45832</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -19929,10 +19921,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A12" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -19962,10 +19952,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A13" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -19995,10 +19983,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A14" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -20028,10 +20014,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A15" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -20061,10 +20045,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A16" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -20094,10 +20076,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A17" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -20127,10 +20107,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A18" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -20160,10 +20138,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A19" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -20193,10 +20169,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A20" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -20226,10 +20200,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A21" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -20259,10 +20231,8 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A22" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -20292,10 +20262,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A23" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -20325,10 +20293,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A24" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -20358,10 +20324,8 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A25" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -20391,10 +20355,8 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A26" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -20424,10 +20386,8 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A27" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -20457,10 +20417,8 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A28" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -20490,10 +20448,8 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2025-10-15</t>
-        </is>
+      <c r="A29" s="1" t="n">
+        <v>45945</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -20929,10 +20885,8 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>2025-10-16</t>
-        </is>
+      <c r="A44" s="1" t="n">
+        <v>45946</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -20962,10 +20916,8 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>2025-10-16</t>
-        </is>
+      <c r="A45" s="1" t="n">
+        <v>45946</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -20995,10 +20947,8 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>2025-10-16</t>
-        </is>
+      <c r="A46" s="1" t="n">
+        <v>45946</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -21028,10 +20978,8 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>2025-10-16</t>
-        </is>
+      <c r="A47" s="1" t="n">
+        <v>45946</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -21061,10 +21009,8 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>2026-02-26</t>
-        </is>
+      <c r="A48" s="1" t="n">
+        <v>46079</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -21094,10 +21040,8 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>2026-02-26</t>
-        </is>
+      <c r="A49" s="1" t="n">
+        <v>46079</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -21127,10 +21071,8 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>2026-04-14</t>
-        </is>
+      <c r="A50" s="1" t="n">
+        <v>46126</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -21160,10 +21102,8 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>2025-10-16</t>
-        </is>
+      <c r="A51" s="1" t="n">
+        <v>45946</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -21193,10 +21133,8 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>2025-10-16</t>
-        </is>
+      <c r="A52" s="1" t="n">
+        <v>45946</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -21226,10 +21164,8 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>2025-10-16</t>
-        </is>
+      <c r="A53" s="1" t="n">
+        <v>45946</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -21259,10 +21195,8 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>2025-10-16</t>
-        </is>
+      <c r="A54" s="1" t="n">
+        <v>45946</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -21292,10 +21226,8 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>2026-02-24</t>
-        </is>
+      <c r="A55" s="1" t="n">
+        <v>46077</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -21325,10 +21257,8 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>2026-02-24</t>
-        </is>
+      <c r="A56" s="1" t="n">
+        <v>46077</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -21358,10 +21288,8 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>2026-02-24</t>
-        </is>
+      <c r="A57" s="1" t="n">
+        <v>46077</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -21391,10 +21319,8 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>2026-02-24</t>
-        </is>
+      <c r="A58" s="1" t="n">
+        <v>46077</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -24295,10 +24221,8 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
+      <c r="A158" s="1" t="n">
+        <v>46161</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -24328,10 +24252,8 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
+      <c r="A159" s="1" t="n">
+        <v>46161</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Seguimiento de cuentas · LS · 2026-08-19 14:54
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -24247,7 +24247,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Pedido de apertura</t>
+          <t>Pedido de apertura. 19/08 consulta estado</t>
         </is>
       </c>
     </row>
@@ -24278,7 +24278,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>Pedido de apertura</t>
+          <t>Pedido de apertura. 19/08 consulta estado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Seguimiento de cuentas · LS · 2026-08-19 15:32
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G601"/>
+  <dimension ref="A1:G602"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19558,6 +19558,39 @@
         </is>
       </c>
       <c r="G601" t="inlineStr"/>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>Comitente</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Banco de Córdoba</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Novus Retorno Total</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr"/>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>Pedido de apertura por mail</t>
+        </is>
+      </c>
+      <c r="G602" t="inlineStr">
+        <is>
+          <t>Aguardamos confirmacion</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Seguimiento de cuentas · LS · 2026-08-21 15:14
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -19578,19 +19578,15 @@
       <c r="D602" t="inlineStr"/>
       <c r="E602" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Abierta</t>
         </is>
       </c>
       <c r="F602" t="inlineStr">
         <is>
-          <t>Pedido de apertura por mail</t>
-        </is>
-      </c>
-      <c r="G602" t="inlineStr">
-        <is>
-          <t>Aguardamos confirmacion</t>
-        </is>
-      </c>
+          <t>Ok para operar.</t>
+        </is>
+      </c>
+      <c r="G602" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Seguimiento de cuentas · LS · 2026-08-21 18:29
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -24331,12 +24331,12 @@
       <c r="E160" t="inlineStr"/>
       <c r="F160" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Abierta</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>Pedido de apertura</t>
+          <t>Falta exención ARCA</t>
         </is>
       </c>
     </row>
@@ -24360,12 +24360,12 @@
       <c r="E161" t="inlineStr"/>
       <c r="F161" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Abierta</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>Pedido de apertura</t>
+          <t>Falta exención ARCA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Seguimiento de cuentas · LS · 2026-09-03 14:30
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -18,10 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -51,9 +48,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G602"/>
+  <dimension ref="A1:G604"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19587,6 +19583,64 @@
         </is>
       </c>
       <c r="G602" t="inlineStr"/>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>Comitente</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Black Toro AM</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Novus Renta Dolar</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr"/>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr"/>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>Falta formulario firmado por Admin y por Depo</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>Comitente</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Black Toro AM</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Novus Gestión</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr"/>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr"/>
+      <c r="G604" t="inlineStr">
+        <is>
+          <t>Falta formulario firmado por Admin y por Depo</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19640,8 +19694,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>45825</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2025-06-17</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -19671,8 +19727,10 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>45825</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-06-17</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -19702,8 +19760,10 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>45825</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-06-17</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -19733,8 +19793,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>45825</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-06-17</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -19764,8 +19826,10 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>46133</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -19795,8 +19859,10 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>45827</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-06-19</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -19826,8 +19892,10 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>45820</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-06-12</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -19857,8 +19925,10 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>45832</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025-06-24</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -19888,8 +19958,10 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>45832</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2025-06-24</t>
+        </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -19919,8 +19991,10 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>45832</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2025-06-24</t>
+        </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -19950,8 +20024,10 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>45945</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -19981,8 +20057,10 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>45945</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -20012,8 +20090,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>45945</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -20043,8 +20123,10 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>45945</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -20074,8 +20156,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>45945</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -20105,8 +20189,10 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>45945</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -20136,8 +20222,10 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
-        <v>45945</v>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -20167,8 +20255,10 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>45945</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -20198,8 +20288,10 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>45945</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -20229,8 +20321,10 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>45945</v>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -20260,8 +20354,10 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>45945</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -20291,8 +20387,10 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>45945</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -20322,8 +20420,10 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>45945</v>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -20353,8 +20453,10 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>45945</v>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -20384,8 +20486,10 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
-        <v>45945</v>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -20415,8 +20519,10 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
-        <v>45945</v>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -20446,8 +20552,10 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
-        <v>45945</v>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -20477,8 +20585,10 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
-        <v>45945</v>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -20914,8 +21024,10 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
-        <v>45946</v>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2025-10-16</t>
+        </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -20945,8 +21057,10 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
-        <v>45946</v>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2025-10-16</t>
+        </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -20976,8 +21090,10 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
-        <v>45946</v>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2025-10-16</t>
+        </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -21007,8 +21123,10 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
-        <v>45946</v>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2025-10-16</t>
+        </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -21038,8 +21156,10 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
-        <v>46079</v>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -21069,8 +21189,10 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
-        <v>46079</v>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -21100,8 +21222,10 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
-        <v>46126</v>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -21131,8 +21255,10 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
-        <v>45946</v>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2025-10-16</t>
+        </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -21162,8 +21288,10 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
-        <v>45946</v>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2025-10-16</t>
+        </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -21193,8 +21321,10 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
-        <v>45946</v>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2025-10-16</t>
+        </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -21224,8 +21354,10 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
-        <v>45946</v>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2025-10-16</t>
+        </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -21255,8 +21387,10 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
-        <v>46077</v>
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -21286,8 +21420,10 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
-        <v>46077</v>
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -21317,8 +21453,10 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
-        <v>46077</v>
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -21348,8 +21486,10 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
-        <v>46077</v>
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -24250,8 +24390,10 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="1" t="n">
-        <v>46161</v>
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -24281,8 +24423,10 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="1" t="n">
-        <v>46161</v>
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Seguimiento de cuentas · LS · 2026-09-03 20:04
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -28593,7 +28593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28932,74 +28932,6 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr"/>
-      <c r="B29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr"/>
-      <c r="B32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr"/>
-      <c r="B33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr"/>
-      <c r="B34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr"/>
-      <c r="B35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr"/>
-      <c r="B36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr"/>
-      <c r="B37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-      <c r="B38" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr"/>
-      <c r="B39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr"/>
-      <c r="B40" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr"/>
-      <c r="B41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr"/>
-      <c r="B43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr"/>
-      <c r="B44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr"/>
-      <c r="B45" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Seguimiento de cuentas · LS · 2026-09-04 16:43
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -705,7 +705,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Novus Gestión II</t>
+          <t>Novus Gestion II</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -781,7 +781,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Estrategia 1172</t>
+          <t>Novus Estrategia</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Estrategia 1172</t>
+          <t>Novus Estrategia</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Estrategia 1172</t>
+          <t>Novus Estrategia</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Novus Gestión</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Novus Gestión</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Novus Gestión</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Novus Gestión II</t>
+          <t>Novus Gestion II</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Novus Ahorro Dólares</t>
+          <t>Novus Ahorro Dolares</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Novus Gestión II</t>
+          <t>Novus Gestion II</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Liquidez Plus 1171</t>
+          <t>Novus Liquidez Plus</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Liquidez </t>
+          <t>Novus Liquidez</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3081,7 +3081,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Valor 1174</t>
+          <t>Novus Valor</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Renta Balanceado 1260</t>
+          <t>Novus Renta Balanceado</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Balanceado 1259</t>
+          <t>Novus Balanceado</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Novus Income</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Novus Performance</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3291,7 +3291,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Renta Mixta</t>
+          <t>Novus Renta Mixta</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Renta Fija</t>
+          <t>Novus Renta Fija</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3375,7 +3375,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Multiestrategia</t>
+          <t>Novus Multiestrategia</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -4297,7 +4297,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D102" t="inlineStr"/>
@@ -4555,7 +4555,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D109" t="inlineStr"/>
@@ -4589,7 +4589,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D110" t="inlineStr"/>
@@ -4623,7 +4623,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Liquidez Plus 1171</t>
+          <t>Novus Liquidez Plus</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -4665,7 +4665,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D112" t="inlineStr"/>
@@ -4699,7 +4699,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Liquidez</t>
+          <t>Novus Liquidez</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -4741,7 +4741,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Valor 1174</t>
+          <t>Novus Valor</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Renta Balanceado 1260</t>
+          <t>Novus Renta Balanceado</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -4825,7 +4825,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Balanceado 1259</t>
+          <t>Novus Balanceado</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -4867,7 +4867,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Novus Income</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -4909,7 +4909,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Novus Performance</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -4951,7 +4951,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Renta Mixta</t>
+          <t>Novus Renta Mixta</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -4993,7 +4993,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Renta Fija</t>
+          <t>Novus Renta Fija</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -5035,7 +5035,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Multiestrategia</t>
+          <t>Novus Multiestrategia</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -5077,7 +5077,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D122" t="inlineStr"/>
@@ -5149,7 +5149,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Novus Renta Dólar</t>
+          <t>Novus Renta Dolar</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -5191,7 +5191,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D125" t="inlineStr"/>
@@ -5225,7 +5225,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D126" t="inlineStr"/>
@@ -5255,7 +5255,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D127" t="inlineStr"/>
@@ -5361,7 +5361,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Novus Income</t>
+          <t>Novus Income</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -5399,7 +5399,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D131" t="inlineStr"/>
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D138" t="inlineStr"/>
@@ -5901,7 +5901,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t xml:space="preserve">Performance </t>
+          <t>Novus Performance</t>
         </is>
       </c>
       <c r="D146" t="inlineStr"/>
@@ -6079,7 +6079,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D151" t="inlineStr"/>
@@ -6109,7 +6109,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D152" t="inlineStr"/>
@@ -6139,7 +6139,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D153" t="inlineStr"/>
@@ -6169,7 +6169,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D154" t="inlineStr"/>
@@ -6351,7 +6351,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D159" t="inlineStr"/>
@@ -6575,7 +6575,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -6955,7 +6955,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D175" t="inlineStr"/>
@@ -7213,7 +7213,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -7861,7 +7861,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D200" t="inlineStr"/>
@@ -8271,7 +8271,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D211" t="inlineStr"/>
@@ -8427,7 +8427,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D215" t="inlineStr"/>
@@ -8457,7 +8457,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D216" t="inlineStr"/>
@@ -8525,7 +8525,7 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D218" t="inlineStr"/>
@@ -8555,7 +8555,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D219" t="inlineStr"/>
@@ -8585,7 +8585,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D220" t="inlineStr"/>
@@ -8619,7 +8619,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D221" t="inlineStr"/>
@@ -8649,7 +8649,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D222" t="inlineStr"/>
@@ -8679,7 +8679,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D223" t="inlineStr"/>
@@ -8823,7 +8823,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D227" t="inlineStr"/>
@@ -9123,7 +9123,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -9389,7 +9389,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="D242" t="inlineStr"/>
@@ -9427,7 +9427,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Liquidez Plus 1171</t>
+          <t>Novus Liquidez Plus</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -9469,7 +9469,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Novus Gestion Plus</t>
+          <t>Novus Gestión Plus</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -9507,7 +9507,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Liquidez</t>
+          <t>Novus Liquidez</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -9549,7 +9549,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Valor 1174</t>
+          <t>Novus Valor</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -9591,7 +9591,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Renta Balanceado 1260</t>
+          <t>Novus Renta Balanceado</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -9633,7 +9633,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Balanceado 1259</t>
+          <t>Novus Balanceado</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -9675,7 +9675,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Novus Income</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -9717,7 +9717,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Novus Performance</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -9759,7 +9759,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Renta Mixta</t>
+          <t>Novus Renta Mixta</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -9801,7 +9801,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Renta Fija</t>
+          <t>Novus Renta Fija</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -9843,7 +9843,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Multiestrategia</t>
+          <t>Novus Multiestrategia</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -9885,7 +9885,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Novus Gestion Plus</t>
+          <t>Novus Gestión Plus</t>
         </is>
       </c>
       <c r="D254" t="inlineStr"/>
@@ -9961,7 +9961,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Novus Renta Dólar</t>
+          <t>Novus Renta Dolar</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -10003,7 +10003,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Novus Gestion Plus</t>
+          <t>Novus Gestión Plus</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -10041,7 +10041,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>NOVUS LIQUIDEZ PLUS</t>
+          <t>Novus Liquidez Plus</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>NOVUS LIQUIDEZ</t>
+          <t>Novus Liquidez</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -10117,7 +10117,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>NOVUS ESTRATEGIA</t>
+          <t>Novus Estrategia</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>NOVUS VALOR</t>
+          <t>Novus Valor</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -10193,7 +10193,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Novus Gestion Plus</t>
+          <t>Novus Gestión Plus</t>
         </is>
       </c>
       <c r="D262" t="inlineStr"/>
@@ -10227,7 +10227,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>NOVUS INCOME</t>
+          <t>Novus Income</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
@@ -10265,7 +10265,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>NOVUS MULTIESTRATEGIA</t>
+          <t>Novus Multiestrategia</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -10303,7 +10303,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>NOVUS RENTA MIXTA</t>
+          <t>Novus Renta Mixta</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -10341,7 +10341,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>NOVUS PERFORMANCE</t>
+          <t>Novus Performance</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -10379,7 +10379,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>NOVUS RENTA FIJA</t>
+          <t>Novus Renta Fija</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
@@ -10417,7 +10417,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Novus Gestion Plus</t>
+          <t>Novus Gestión Plus</t>
         </is>
       </c>
       <c r="D268" t="inlineStr"/>
@@ -10447,7 +10447,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>NOVUS GESTIÓN II</t>
+          <t>Novus Gestion II</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -10485,7 +10485,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>NOVUS RENTA CAPITAL</t>
+          <t>Novus Renta Capital</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
@@ -10523,7 +10523,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>NOVUS CAPITAL</t>
+          <t>Novus Capital</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
@@ -10561,7 +10561,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>NOVUS AHORRO DÓLARES</t>
+          <t>Novus Ahorro Dolares</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -10599,7 +10599,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Novus Gestion Plus</t>
+          <t>Novus Gestión Plus</t>
         </is>
       </c>
       <c r="D273" t="inlineStr"/>
@@ -10819,7 +10819,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Novus Gestion Plus</t>
+          <t>Novus Gestión Plus</t>
         </is>
       </c>
       <c r="D279" t="inlineStr"/>
@@ -10925,7 +10925,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Novus Ahorro Dólares</t>
+          <t>Novus Ahorro Dolares</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -11001,7 +11001,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Novus Gestión II</t>
+          <t>Novus Gestion II</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -11077,7 +11077,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Novus Gestion Plus</t>
+          <t>Novus Gestión Plus</t>
         </is>
       </c>
       <c r="D286" t="inlineStr"/>
@@ -11301,7 +11301,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Novus Gestion Plus</t>
+          <t>Novus Gestión Plus</t>
         </is>
       </c>
       <c r="D292" t="inlineStr"/>
@@ -11597,7 +11597,7 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Novus Gestion Plus</t>
+          <t>Novus Gestión Plus</t>
         </is>
       </c>
       <c r="D300" t="inlineStr"/>
@@ -11711,7 +11711,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Novus Gestion</t>
+          <t>Novus Gestión</t>
         </is>
       </c>
       <c r="D303" t="inlineStr"/>
@@ -11977,7 +11977,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Novus Gestion Plus</t>
+          <t>Novus Gestión Plus</t>
         </is>
       </c>
       <c r="D310" t="inlineStr"/>
@@ -12339,7 +12339,7 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Novus Gestion Plus</t>
+          <t>Novus Gestión Plus</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
@@ -12867,7 +12867,7 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Novus Gestion</t>
+          <t>Novus Gestión</t>
         </is>
       </c>
       <c r="D333" t="inlineStr"/>
@@ -13219,7 +13219,7 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>Novus Gestion</t>
+          <t>Novus Gestión</t>
         </is>
       </c>
       <c r="D343" t="inlineStr"/>
@@ -13253,7 +13253,7 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Novus Gestion</t>
+          <t>Novus Gestión</t>
         </is>
       </c>
       <c r="D344" t="inlineStr"/>
@@ -15023,7 +15023,7 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>Novus PYME FCI Abierto PyMES</t>
+          <t>Novus PyME FCI Abierto PyMES</t>
         </is>
       </c>
       <c r="D393" t="inlineStr">
@@ -15103,7 +15103,7 @@
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>Novus PYME FCI Abierto PyMES</t>
+          <t>Novus PyME FCI Abierto PyMES</t>
         </is>
       </c>
       <c r="D395" t="inlineStr">
@@ -15293,7 +15293,7 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>Novus PYME FCI Abierto PyMES</t>
+          <t>Novus PyME FCI Abierto PyMES</t>
         </is>
       </c>
       <c r="D400" t="inlineStr">
@@ -15335,7 +15335,7 @@
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>NOVUS PYME FCI ABIERTO PYMES</t>
+          <t>Novus PyME FCI Abierto PyMES</t>
         </is>
       </c>
       <c r="D401" t="inlineStr">
@@ -15525,7 +15525,7 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t xml:space="preserve">Novus Gestion </t>
+          <t>Novus Gestión</t>
         </is>
       </c>
       <c r="D406" t="inlineStr">
@@ -16549,7 +16549,7 @@
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>Novus Gestion</t>
+          <t>Novus Gestión</t>
         </is>
       </c>
       <c r="D434" t="inlineStr"/>
@@ -16855,7 +16855,7 @@
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>Novus renta fIJA</t>
+          <t>Novus Renta Fija</t>
         </is>
       </c>
       <c r="D443" t="inlineStr"/>
@@ -18955,7 +18955,7 @@
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>NOVUS RENTA BALANCEADO</t>
+          <t>Novus Renta Balanceado</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
@@ -21213,7 +21213,7 @@
       </c>
       <c r="C566" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Liquidez Plus FCI</t>
+          <t>Novus Liquidez Plus</t>
         </is>
       </c>
       <c r="D566" t="inlineStr"/>
@@ -21289,7 +21289,7 @@
       </c>
       <c r="C568" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Estrategia FCI</t>
+          <t>Novus Estrategia</t>
         </is>
       </c>
       <c r="D568" t="inlineStr"/>
@@ -21365,7 +21365,7 @@
       </c>
       <c r="C570" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Renta Balanceado FCI</t>
+          <t>Novus Renta Balanceado</t>
         </is>
       </c>
       <c r="D570" t="inlineStr"/>
@@ -21403,7 +21403,7 @@
       </c>
       <c r="C571" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Balanceado FCI</t>
+          <t>Novus Balanceado</t>
         </is>
       </c>
       <c r="D571" t="inlineStr"/>
@@ -21517,7 +21517,7 @@
       </c>
       <c r="C574" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Renta Mixta FCI</t>
+          <t>Novus Renta Mixta</t>
         </is>
       </c>
       <c r="D574" t="inlineStr"/>
@@ -21555,7 +21555,7 @@
       </c>
       <c r="C575" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Performance FCI</t>
+          <t>Novus Performance</t>
         </is>
       </c>
       <c r="D575" t="inlineStr"/>
@@ -21593,7 +21593,7 @@
       </c>
       <c r="C576" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Renta Fija FCI</t>
+          <t>Novus Renta Fija</t>
         </is>
       </c>
       <c r="D576" t="inlineStr"/>
@@ -21745,7 +21745,7 @@
       </c>
       <c r="C580" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Capital FCI</t>
+          <t>Novus Capital</t>
         </is>
       </c>
       <c r="D580" t="inlineStr"/>
@@ -21821,7 +21821,7 @@
       </c>
       <c r="C582" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Liquidez Plus FCI</t>
+          <t>Novus Liquidez Plus</t>
         </is>
       </c>
       <c r="D582" t="inlineStr">
@@ -21859,7 +21859,7 @@
       </c>
       <c r="C583" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Estrategia FCI</t>
+          <t>Novus Estrategia</t>
         </is>
       </c>
       <c r="D583" t="inlineStr">
@@ -21973,7 +21973,7 @@
       </c>
       <c r="C586" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Renta Balanceado FCI</t>
+          <t>Novus Renta Balanceado</t>
         </is>
       </c>
       <c r="D586" t="inlineStr">
@@ -22011,7 +22011,7 @@
       </c>
       <c r="C587" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Balanceado FCI</t>
+          <t>Novus Balanceado</t>
         </is>
       </c>
       <c r="D587" t="inlineStr">
@@ -22163,7 +22163,7 @@
       </c>
       <c r="C591" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Performance FCI</t>
+          <t>Novus Performance</t>
         </is>
       </c>
       <c r="D591" t="inlineStr">
@@ -22201,7 +22201,7 @@
       </c>
       <c r="C592" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Renta Fija FCI</t>
+          <t>Novus Renta Fija</t>
         </is>
       </c>
       <c r="D592" t="inlineStr">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="C593" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Renta Mixta FCI</t>
+          <t>Novus Renta Mixta</t>
         </is>
       </c>
       <c r="D593" t="inlineStr">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="C596" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Capital FCI</t>
+          <t>Novus Capital</t>
         </is>
       </c>
       <c r="D596" t="inlineStr">

</xml_diff>

<commit_message>
Seguimiento de cuentas · LS · 2026-09-04 16:44
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -5765,7 +5765,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t xml:space="preserve">Liquidez Plus </t>
+          <t>Novus Liquidez Plus</t>
         </is>
       </c>
       <c r="D142" t="inlineStr"/>
@@ -5799,7 +5799,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Valor</t>
+          <t>Novus Valor</t>
         </is>
       </c>
       <c r="D143" t="inlineStr"/>
@@ -5833,7 +5833,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Estrategia</t>
+          <t>Novus Estrategia</t>
         </is>
       </c>
       <c r="D144" t="inlineStr"/>
@@ -5935,7 +5935,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Capital USDM</t>
+          <t>Novus Capital</t>
         </is>
       </c>
       <c r="D147" t="inlineStr"/>
@@ -21251,7 +21251,7 @@
       </c>
       <c r="C567" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Liquidez FCI</t>
+          <t>Novus Liquidez</t>
         </is>
       </c>
       <c r="D567" t="inlineStr"/>
@@ -21479,7 +21479,7 @@
       </c>
       <c r="C573" t="inlineStr">
         <is>
-          <t>BVSA SD Novus MultiestrategiaFCI</t>
+          <t>Novus Multiestrategia</t>
         </is>
       </c>
       <c r="D573" t="inlineStr"/>
@@ -21631,7 +21631,7 @@
       </c>
       <c r="C577" t="inlineStr">
         <is>
-          <t>BVSA SD Novus PyME FCI Abierto PyMES FCI</t>
+          <t>Novus PyME FCI Abierto PyMES</t>
         </is>
       </c>
       <c r="D577" t="inlineStr"/>
@@ -21669,7 +21669,7 @@
       </c>
       <c r="C578" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Gestion II FCI</t>
+          <t>Novus Gestion II</t>
         </is>
       </c>
       <c r="D578" t="inlineStr"/>
@@ -21707,7 +21707,7 @@
       </c>
       <c r="C579" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Renta Capital FCI</t>
+          <t>Novus Renta Capital</t>
         </is>
       </c>
       <c r="D579" t="inlineStr"/>
@@ -21897,7 +21897,7 @@
       </c>
       <c r="C584" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Liquidez Fondo de Dinero FCI</t>
+          <t>Novus Liquidez</t>
         </is>
       </c>
       <c r="D584" t="inlineStr">
@@ -22049,7 +22049,7 @@
       </c>
       <c r="C588" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Income FCI</t>
+          <t>Novus Income</t>
         </is>
       </c>
       <c r="D588" t="inlineStr">
@@ -22125,7 +22125,7 @@
       </c>
       <c r="C590" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Multiestrategia FCI</t>
+          <t>Novus Multiestrategia</t>
         </is>
       </c>
       <c r="D590" t="inlineStr">
@@ -22277,7 +22277,7 @@
       </c>
       <c r="C594" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Renta Dolar FCI</t>
+          <t>Novus Renta Dolar</t>
         </is>
       </c>
       <c r="D594" t="inlineStr">
@@ -22315,7 +22315,7 @@
       </c>
       <c r="C595" t="inlineStr">
         <is>
-          <t>BVSA SD Novus PYME FCI Abierto PyMES</t>
+          <t>Novus PyME FCI Abierto PyMES</t>
         </is>
       </c>
       <c r="D595" t="inlineStr">
@@ -22391,7 +22391,7 @@
       </c>
       <c r="C597" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Renta Variable FCI</t>
+          <t>Novus Renta Variable</t>
         </is>
       </c>
       <c r="D597" t="inlineStr">

</xml_diff>

<commit_message>
Seguimiento de cuentas · LS · 2026-09-04 16:46
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -5867,7 +5867,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Gestión II</t>
+          <t>Novus Gestion II</t>
         </is>
       </c>
       <c r="D145" t="inlineStr"/>
@@ -5969,7 +5969,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Gestión II</t>
+          <t>Novus Gestion II</t>
         </is>
       </c>
       <c r="D148" t="inlineStr"/>
@@ -21327,7 +21327,7 @@
       </c>
       <c r="C569" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Valor FCI</t>
+          <t>Novus Valor</t>
         </is>
       </c>
       <c r="D569" t="inlineStr"/>
@@ -21441,7 +21441,7 @@
       </c>
       <c r="C572" t="inlineStr">
         <is>
-          <t>BVSA SD Novus IncomeFCI</t>
+          <t>Novus Income</t>
         </is>
       </c>
       <c r="D572" t="inlineStr"/>
@@ -21783,7 +21783,7 @@
       </c>
       <c r="C581" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Ahorro Dolares FCI</t>
+          <t>Novus Ahorro Dolares</t>
         </is>
       </c>
       <c r="D581" t="inlineStr"/>
@@ -21935,7 +21935,7 @@
       </c>
       <c r="C585" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Valor FCI</t>
+          <t>Novus Valor</t>
         </is>
       </c>
       <c r="D585" t="inlineStr">
@@ -22087,7 +22087,7 @@
       </c>
       <c r="C589" t="inlineStr">
         <is>
-          <t>BVSA SD Novus Gestion FCI</t>
+          <t>Novus Gestión</t>
         </is>
       </c>
       <c r="D589" t="inlineStr">
@@ -22429,7 +22429,7 @@
       </c>
       <c r="C598" t="inlineStr">
         <is>
-          <t>BVSA SD NOVUS GESTION PLUS</t>
+          <t>Novus Gestión Plus</t>
         </is>
       </c>
       <c r="D598" t="inlineStr">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="C599" t="inlineStr">
         <is>
-          <t>BVSA SD NOVUS CRECIMIENTO</t>
+          <t>Novus Crecimiento</t>
         </is>
       </c>
       <c r="D599" t="inlineStr">

</xml_diff>

<commit_message>
Seguimiento de cuentas · LS · 2026-09-04 16:48
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -28593,7 +28593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28932,6 +28932,14 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Novus Global I</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Seguimiento de cuentas · LS · 2026-09-04 18:43
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -22677,7 +22677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J161"/>
+  <dimension ref="A1:J163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28581,6 +28581,74 @@
       </c>
       <c r="I161" t="inlineStr"/>
       <c r="J161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Remunerada</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Banco Supervielle</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Novus PyME FCI Abierto PyMES</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr"/>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr"/>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>1. Inicio / Solicitud</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Remunerada</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Banco Supervielle</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Novus Renta Variable</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr"/>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr"/>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>1. Inicio / Solicitud</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr"/>
+      <c r="J163" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>